<commit_message>
Additional Retest cases commit
</commit_message>
<xml_diff>
--- a/ParaBankAutomationFramework/src/main/java/ParaBank-TestData/ParaBank-TestDataExcelSheet.xlsx
+++ b/ParaBankAutomationFramework/src/main/java/ParaBank-TestData/ParaBank-TestDataExcelSheet.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="29">
   <si>
     <t>password</t>
   </si>
@@ -76,7 +76,31 @@
     <t>JJ Nagar, LIC Colony</t>
   </si>
   <si>
-    <t>katty</t>
+    <t>Retest - TestData</t>
+  </si>
+  <si>
+    <t>User 2</t>
+  </si>
+  <si>
+    <t>User 1</t>
+  </si>
+  <si>
+    <t>InitialAccountID</t>
+  </si>
+  <si>
+    <t>16230</t>
+  </si>
+  <si>
+    <t>16341</t>
+  </si>
+  <si>
+    <t>16452</t>
+  </si>
+  <si>
+    <t>tom</t>
+  </si>
+  <si>
+    <t>jerry</t>
   </si>
 </sst>
 </file>
@@ -86,7 +110,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0;[Red]0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -98,6 +122,22 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -124,7 +164,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -132,6 +172,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -434,30 +481,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="28.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -465,7 +515,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -473,7 +523,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -481,7 +531,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -489,7 +539,7 @@
         <v>613001</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -497,7 +547,7 @@
         <v>98765</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -505,36 +555,39 @@
         <v>12345</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>0</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -542,7 +595,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -550,7 +603,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -558,7 +611,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -566,21 +619,93 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="B19" s="2"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
+      <c r="C19" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>2</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="4"/>
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B27" s="1"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B28" s="1"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B29" s="1"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B30" s="1"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B31" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>